<commit_message>
Resumo→Envio; nova guia Empresa (PLR = Resultado da Empresa × Resultado do Book × 1,6) com tabela do book e faixa da fórmula; Cargo/Responsável como lista suspensa multisseleção; demo com 'Resultado da Empresa' fictício (peso 0); cache-bust
</commit_message>
<xml_diff>
--- a/demo-BD-BOOK.xlsx
+++ b/demo-BD-BOOK.xlsx
@@ -426,7 +426,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W95"/>
+  <dimension ref="A1:W101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,40 +457,40 @@
         <v>Desafio</v>
       </c>
       <c r="J1" s="1">
-        <v>45321.87467592592</v>
+        <v>45321.875</v>
       </c>
       <c r="K1" s="1">
-        <v>45350.87467592592</v>
+        <v>45350.875</v>
       </c>
       <c r="L1" s="1">
-        <v>45381.87467592592</v>
+        <v>45381.875</v>
       </c>
       <c r="M1" s="1">
-        <v>45411.87467592592</v>
+        <v>45411.875</v>
       </c>
       <c r="N1" s="1">
-        <v>45442.87467592592</v>
+        <v>45442.875</v>
       </c>
       <c r="O1" s="1">
-        <v>45472.87467592592</v>
+        <v>45472.875</v>
       </c>
       <c r="P1" s="1">
-        <v>45503.87467592592</v>
+        <v>45503.875</v>
       </c>
       <c r="Q1" s="1">
-        <v>45534.87467592592</v>
+        <v>45534.875</v>
       </c>
       <c r="R1" s="1">
-        <v>45564.87467592592</v>
+        <v>45564.875</v>
       </c>
       <c r="S1" s="1">
-        <v>45595.87467592592</v>
+        <v>45595.875</v>
       </c>
       <c r="T1" s="1">
-        <v>45625.87467592592</v>
+        <v>45625.875</v>
       </c>
       <c r="U1" s="1">
-        <v>45656.87467592592</v>
+        <v>45656.875</v>
       </c>
       <c r="V1" t="str">
         <v>Acumulado</v>
@@ -7173,16 +7173,442 @@
         <v>2026</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>CSC</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Book Geral CSC</v>
+      </c>
+      <c r="C96" t="str">
+        <v>-</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E96" t="str">
+        <v>%</v>
+      </c>
+      <c r="F96">
+        <v>0</v>
+      </c>
+      <c r="G96" t="str">
+        <v>h</v>
+      </c>
+      <c r="H96">
+        <v>0.9999</v>
+      </c>
+      <c r="I96" t="str">
+        <v>-</v>
+      </c>
+      <c r="J96">
+        <v>100</v>
+      </c>
+      <c r="K96">
+        <v>100</v>
+      </c>
+      <c r="L96">
+        <v>100</v>
+      </c>
+      <c r="M96">
+        <v>100</v>
+      </c>
+      <c r="N96">
+        <v>100</v>
+      </c>
+      <c r="O96">
+        <v>100</v>
+      </c>
+      <c r="P96">
+        <v>100</v>
+      </c>
+      <c r="Q96">
+        <v>100</v>
+      </c>
+      <c r="R96">
+        <v>100</v>
+      </c>
+      <c r="S96">
+        <v>100</v>
+      </c>
+      <c r="T96">
+        <v>100</v>
+      </c>
+      <c r="U96">
+        <v>100</v>
+      </c>
+      <c r="V96">
+        <v>100</v>
+      </c>
+      <c r="W96">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>MIG</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Book Geral MIG</v>
+      </c>
+      <c r="C97" t="str">
+        <v>0</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E97" t="str">
+        <v>%</v>
+      </c>
+      <c r="F97">
+        <v>0</v>
+      </c>
+      <c r="G97" t="str">
+        <v>h</v>
+      </c>
+      <c r="H97">
+        <v>0.9999</v>
+      </c>
+      <c r="I97" t="str">
+        <v>-</v>
+      </c>
+      <c r="J97">
+        <v>100</v>
+      </c>
+      <c r="K97">
+        <v>100</v>
+      </c>
+      <c r="L97">
+        <v>100</v>
+      </c>
+      <c r="M97">
+        <v>100</v>
+      </c>
+      <c r="N97">
+        <v>100</v>
+      </c>
+      <c r="O97">
+        <v>100</v>
+      </c>
+      <c r="P97">
+        <v>100</v>
+      </c>
+      <c r="Q97">
+        <v>100</v>
+      </c>
+      <c r="R97">
+        <v>100</v>
+      </c>
+      <c r="S97">
+        <v>100</v>
+      </c>
+      <c r="T97">
+        <v>100</v>
+      </c>
+      <c r="U97">
+        <v>100</v>
+      </c>
+      <c r="V97">
+        <v>100</v>
+      </c>
+      <c r="W97">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>MML</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Book Geral MML</v>
+      </c>
+      <c r="C98" t="str">
+        <v>-</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E98" t="str">
+        <v>%</v>
+      </c>
+      <c r="F98">
+        <v>0</v>
+      </c>
+      <c r="G98" t="str">
+        <v>h</v>
+      </c>
+      <c r="H98">
+        <v>0.9999</v>
+      </c>
+      <c r="I98" t="str">
+        <v>-</v>
+      </c>
+      <c r="J98">
+        <v>100</v>
+      </c>
+      <c r="K98">
+        <v>100</v>
+      </c>
+      <c r="L98">
+        <v>100</v>
+      </c>
+      <c r="M98">
+        <v>100</v>
+      </c>
+      <c r="N98">
+        <v>100</v>
+      </c>
+      <c r="O98">
+        <v>100</v>
+      </c>
+      <c r="P98">
+        <v>100</v>
+      </c>
+      <c r="Q98">
+        <v>100</v>
+      </c>
+      <c r="R98">
+        <v>100</v>
+      </c>
+      <c r="S98">
+        <v>100</v>
+      </c>
+      <c r="T98">
+        <v>100</v>
+      </c>
+      <c r="U98">
+        <v>100</v>
+      </c>
+      <c r="V98">
+        <v>100</v>
+      </c>
+      <c r="W98">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>CSC</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Book Geral CSC</v>
+      </c>
+      <c r="C99" t="str">
+        <v>-</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E99" t="str">
+        <v>%</v>
+      </c>
+      <c r="F99">
+        <v>0</v>
+      </c>
+      <c r="G99" t="str">
+        <v>h</v>
+      </c>
+      <c r="H99">
+        <v>0.9999</v>
+      </c>
+      <c r="I99" t="str">
+        <v>-</v>
+      </c>
+      <c r="J99">
+        <v>100</v>
+      </c>
+      <c r="K99">
+        <v>100</v>
+      </c>
+      <c r="L99">
+        <v>100</v>
+      </c>
+      <c r="M99">
+        <v>100</v>
+      </c>
+      <c r="N99">
+        <v>100</v>
+      </c>
+      <c r="O99">
+        <v>100</v>
+      </c>
+      <c r="P99">
+        <v>100</v>
+      </c>
+      <c r="Q99">
+        <v>100</v>
+      </c>
+      <c r="R99">
+        <v>100</v>
+      </c>
+      <c r="S99">
+        <v>100</v>
+      </c>
+      <c r="T99">
+        <v>100</v>
+      </c>
+      <c r="U99">
+        <v>100</v>
+      </c>
+      <c r="V99">
+        <v>100</v>
+      </c>
+      <c r="W99">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>MIG</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Book Geral MIG</v>
+      </c>
+      <c r="C100" t="str">
+        <v>0</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E100" t="str">
+        <v>%</v>
+      </c>
+      <c r="F100">
+        <v>0</v>
+      </c>
+      <c r="G100" t="str">
+        <v>h</v>
+      </c>
+      <c r="H100">
+        <v>0.9999</v>
+      </c>
+      <c r="I100" t="str">
+        <v>-</v>
+      </c>
+      <c r="J100">
+        <v>100</v>
+      </c>
+      <c r="K100">
+        <v>100</v>
+      </c>
+      <c r="L100">
+        <v>100</v>
+      </c>
+      <c r="M100">
+        <v>100</v>
+      </c>
+      <c r="N100">
+        <v>100</v>
+      </c>
+      <c r="O100">
+        <v>100</v>
+      </c>
+      <c r="P100">
+        <v>100</v>
+      </c>
+      <c r="Q100">
+        <v>100</v>
+      </c>
+      <c r="R100">
+        <v>100</v>
+      </c>
+      <c r="S100">
+        <v>100</v>
+      </c>
+      <c r="T100">
+        <v>100</v>
+      </c>
+      <c r="U100">
+        <v>100</v>
+      </c>
+      <c r="V100">
+        <v>100</v>
+      </c>
+      <c r="W100">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>MML</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Book Geral MML</v>
+      </c>
+      <c r="C101" t="str">
+        <v>-</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E101" t="str">
+        <v>%</v>
+      </c>
+      <c r="F101">
+        <v>0</v>
+      </c>
+      <c r="G101" t="str">
+        <v>h</v>
+      </c>
+      <c r="H101">
+        <v>0.9999</v>
+      </c>
+      <c r="I101" t="str">
+        <v>-</v>
+      </c>
+      <c r="J101">
+        <v>100</v>
+      </c>
+      <c r="K101">
+        <v>100</v>
+      </c>
+      <c r="L101">
+        <v>100</v>
+      </c>
+      <c r="M101">
+        <v>100</v>
+      </c>
+      <c r="N101">
+        <v>100</v>
+      </c>
+      <c r="O101">
+        <v>100</v>
+      </c>
+      <c r="P101">
+        <v>100</v>
+      </c>
+      <c r="Q101">
+        <v>100</v>
+      </c>
+      <c r="R101">
+        <v>100</v>
+      </c>
+      <c r="S101">
+        <v>100</v>
+      </c>
+      <c r="T101">
+        <v>100</v>
+      </c>
+      <c r="U101">
+        <v>100</v>
+      </c>
+      <c r="V101">
+        <v>100</v>
+      </c>
+      <c r="W101">
+        <v>2026</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W95"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W101"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W95"/>
+  <dimension ref="A1:W101"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7213,40 +7639,40 @@
         <v>Desafio</v>
       </c>
       <c r="J1" s="1">
-        <v>45321.87467592592</v>
+        <v>45321.875</v>
       </c>
       <c r="K1" s="1">
-        <v>45350.87467592592</v>
+        <v>45350.875</v>
       </c>
       <c r="L1" s="1">
-        <v>45381.87467592592</v>
+        <v>45381.875</v>
       </c>
       <c r="M1" s="1">
-        <v>45411.87467592592</v>
+        <v>45411.875</v>
       </c>
       <c r="N1" s="1">
-        <v>45442.87467592592</v>
+        <v>45442.875</v>
       </c>
       <c r="O1" s="1">
-        <v>45472.87467592592</v>
+        <v>45472.875</v>
       </c>
       <c r="P1" s="1">
-        <v>45503.87467592592</v>
+        <v>45503.875</v>
       </c>
       <c r="Q1" s="1">
-        <v>45534.87467592592</v>
+        <v>45534.875</v>
       </c>
       <c r="R1" s="1">
-        <v>45564.87467592592</v>
+        <v>45564.875</v>
       </c>
       <c r="S1" s="1">
-        <v>45595.87467592592</v>
+        <v>45595.875</v>
       </c>
       <c r="T1" s="1">
-        <v>45625.87467592592</v>
+        <v>45625.875</v>
       </c>
       <c r="U1" s="1">
-        <v>45656.87467592592</v>
+        <v>45656.875</v>
       </c>
       <c r="V1" t="str">
         <v>Acumulado</v>
@@ -13365,9 +13791,399 @@
         <v>2026</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>CSC</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Book Geral CSC</v>
+      </c>
+      <c r="C96" t="str">
+        <v>-</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E96" t="str">
+        <v>%</v>
+      </c>
+      <c r="F96">
+        <v>0</v>
+      </c>
+      <c r="G96" t="str">
+        <v>h</v>
+      </c>
+      <c r="H96">
+        <v>0.9999</v>
+      </c>
+      <c r="I96" t="str">
+        <v>-</v>
+      </c>
+      <c r="J96">
+        <v>77.1</v>
+      </c>
+      <c r="K96">
+        <v>84.3</v>
+      </c>
+      <c r="L96">
+        <v>75.1</v>
+      </c>
+      <c r="M96">
+        <v>77.1</v>
+      </c>
+      <c r="N96">
+        <v>99.7</v>
+      </c>
+      <c r="O96">
+        <v>83.3</v>
+      </c>
+      <c r="P96">
+        <v>99.4</v>
+      </c>
+      <c r="Q96">
+        <v>100.8</v>
+      </c>
+      <c r="R96">
+        <v>77.8</v>
+      </c>
+      <c r="S96">
+        <v>79.5</v>
+      </c>
+      <c r="T96">
+        <v>90.8</v>
+      </c>
+      <c r="U96">
+        <v>78.5</v>
+      </c>
+      <c r="V96">
+        <v>85.28</v>
+      </c>
+      <c r="W96">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>MIG</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Book Geral MIG</v>
+      </c>
+      <c r="C97" t="str">
+        <v>0</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E97" t="str">
+        <v>%</v>
+      </c>
+      <c r="F97">
+        <v>0</v>
+      </c>
+      <c r="G97" t="str">
+        <v>h</v>
+      </c>
+      <c r="H97">
+        <v>0.9999</v>
+      </c>
+      <c r="I97" t="str">
+        <v>-</v>
+      </c>
+      <c r="J97">
+        <v>91.2</v>
+      </c>
+      <c r="K97">
+        <v>84.7</v>
+      </c>
+      <c r="L97">
+        <v>97.1</v>
+      </c>
+      <c r="M97">
+        <v>78.6</v>
+      </c>
+      <c r="N97">
+        <v>75.1</v>
+      </c>
+      <c r="O97">
+        <v>86.8</v>
+      </c>
+      <c r="P97">
+        <v>75</v>
+      </c>
+      <c r="Q97">
+        <v>83.2</v>
+      </c>
+      <c r="R97">
+        <v>86.4</v>
+      </c>
+      <c r="S97">
+        <v>81.3</v>
+      </c>
+      <c r="T97">
+        <v>81.2</v>
+      </c>
+      <c r="U97">
+        <v>79.5</v>
+      </c>
+      <c r="V97">
+        <v>83.34</v>
+      </c>
+      <c r="W97">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>MML</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Book Geral MML</v>
+      </c>
+      <c r="C98" t="str">
+        <v>-</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E98" t="str">
+        <v>%</v>
+      </c>
+      <c r="F98">
+        <v>0</v>
+      </c>
+      <c r="G98" t="str">
+        <v>h</v>
+      </c>
+      <c r="H98">
+        <v>0.9999</v>
+      </c>
+      <c r="I98" t="str">
+        <v>-</v>
+      </c>
+      <c r="J98">
+        <v>87.8</v>
+      </c>
+      <c r="K98">
+        <v>90.6</v>
+      </c>
+      <c r="L98">
+        <v>79.6</v>
+      </c>
+      <c r="M98">
+        <v>87.1</v>
+      </c>
+      <c r="N98">
+        <v>76.3</v>
+      </c>
+      <c r="O98">
+        <v>80.2</v>
+      </c>
+      <c r="P98">
+        <v>75.8</v>
+      </c>
+      <c r="Q98">
+        <v>81.4</v>
+      </c>
+      <c r="R98">
+        <v>78.7</v>
+      </c>
+      <c r="S98">
+        <v>96.1</v>
+      </c>
+      <c r="T98">
+        <v>83.2</v>
+      </c>
+      <c r="U98">
+        <v>99</v>
+      </c>
+      <c r="V98">
+        <v>84.65</v>
+      </c>
+      <c r="W98">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>CSC</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Book Geral CSC</v>
+      </c>
+      <c r="C99" t="str">
+        <v>-</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E99" t="str">
+        <v>%</v>
+      </c>
+      <c r="F99">
+        <v>0</v>
+      </c>
+      <c r="G99" t="str">
+        <v>h</v>
+      </c>
+      <c r="H99">
+        <v>0.9999</v>
+      </c>
+      <c r="I99" t="str">
+        <v>-</v>
+      </c>
+      <c r="J99">
+        <v>92.5</v>
+      </c>
+      <c r="K99">
+        <v>85.9</v>
+      </c>
+      <c r="L99">
+        <v>83.3</v>
+      </c>
+      <c r="M99">
+        <v>93.8</v>
+      </c>
+      <c r="N99">
+        <v>85.5</v>
+      </c>
+      <c r="O99">
+        <v>78.8</v>
+      </c>
+      <c r="P99">
+        <v>97</v>
+      </c>
+      <c r="Q99">
+        <v>78.8</v>
+      </c>
+      <c r="V99">
+        <v>86.95</v>
+      </c>
+      <c r="W99">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>MIG</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Book Geral MIG</v>
+      </c>
+      <c r="C100" t="str">
+        <v>0</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E100" t="str">
+        <v>%</v>
+      </c>
+      <c r="F100">
+        <v>0</v>
+      </c>
+      <c r="G100" t="str">
+        <v>h</v>
+      </c>
+      <c r="H100">
+        <v>0.9999</v>
+      </c>
+      <c r="I100" t="str">
+        <v>-</v>
+      </c>
+      <c r="J100">
+        <v>77.1</v>
+      </c>
+      <c r="K100">
+        <v>89.6</v>
+      </c>
+      <c r="L100">
+        <v>97.2</v>
+      </c>
+      <c r="M100">
+        <v>75.4</v>
+      </c>
+      <c r="N100">
+        <v>84.3</v>
+      </c>
+      <c r="O100">
+        <v>75.9</v>
+      </c>
+      <c r="P100">
+        <v>78.3</v>
+      </c>
+      <c r="Q100">
+        <v>77.1</v>
+      </c>
+      <c r="V100">
+        <v>81.86</v>
+      </c>
+      <c r="W100">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>MML</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Book Geral MML</v>
+      </c>
+      <c r="C101" t="str">
+        <v>-</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Resultado da Empresa</v>
+      </c>
+      <c r="E101" t="str">
+        <v>%</v>
+      </c>
+      <c r="F101">
+        <v>0</v>
+      </c>
+      <c r="G101" t="str">
+        <v>h</v>
+      </c>
+      <c r="H101">
+        <v>0.9999</v>
+      </c>
+      <c r="I101" t="str">
+        <v>-</v>
+      </c>
+      <c r="J101">
+        <v>81.2</v>
+      </c>
+      <c r="K101">
+        <v>75</v>
+      </c>
+      <c r="L101">
+        <v>98.1</v>
+      </c>
+      <c r="M101">
+        <v>80.5</v>
+      </c>
+      <c r="N101">
+        <v>76.2</v>
+      </c>
+      <c r="O101">
+        <v>82.6</v>
+      </c>
+      <c r="P101">
+        <v>81</v>
+      </c>
+      <c r="Q101">
+        <v>92.6</v>
+      </c>
+      <c r="V101">
+        <v>83.4</v>
+      </c>
+      <c r="W101">
+        <v>2026</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W95"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W101"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>